<commit_message>
Update: python interpreter 추가
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a45cc3699792be64/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\errop\aws_inventory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F66D8EE-C5EB-4DA7-9EFF-D3F0E568F645}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B843B88D-8D5F-4D3B-AE23-52C98282B8AD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7930" xr2:uid="{062FBF7F-E507-4C39-941B-5A744C0083F2}"/>
   </bookViews>
@@ -460,7 +460,7 @@
         <v>9</v>
       </c>
       <c r="C2">
-        <v>8080</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
         <v>14</v>
@@ -480,7 +480,7 @@
         <v>10</v>
       </c>
       <c r="C3">
-        <v>8080</v>
+        <v>22</v>
       </c>
       <c r="D3" t="s">
         <v>14</v>
@@ -500,7 +500,7 @@
         <v>11</v>
       </c>
       <c r="C4">
-        <v>8080</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
         <v>14</v>

</xml_diff>